<commit_message>
Ajout complet de l'éditeur UML interactif (classes, séquences, cas d'utilisation, redimensionnement)
</commit_message>
<xml_diff>
--- a/liste_etudiants.xlsx
+++ b/liste_etudiants.xlsx
@@ -418,13 +418,13 @@
         <v>ETU001</v>
       </c>
       <c r="B2" t="str">
-        <v>Diop</v>
+        <v>Sow</v>
       </c>
       <c r="C2" t="str">
-        <v>Moussa</v>
+        <v>Seydina Aliou</v>
       </c>
       <c r="D2" t="str">
-        <v>moussa.diop@example.com</v>
+        <v>seydinaaliousow80@gmail.com</v>
       </c>
     </row>
     <row r="3">

</xml_diff>